<commit_message>
Actualización codigo y comentarios
</commit_message>
<xml_diff>
--- a/data/processed/y_test.xlsx
+++ b/data/processed/y_test.xlsx
@@ -440,12 +440,12 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -455,12 +455,12 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -470,7 +470,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -495,12 +495,12 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -515,7 +515,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -525,12 +525,12 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -540,7 +540,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -550,12 +550,12 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -585,12 +585,12 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -615,22 +615,22 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -645,7 +645,7 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -655,7 +655,7 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -665,7 +665,7 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -680,7 +680,7 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -690,12 +690,12 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
@@ -750,7 +750,7 @@
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="68">
@@ -770,7 +770,7 @@
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -785,17 +785,17 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -810,17 +810,17 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -835,7 +835,7 @@
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -845,27 +845,27 @@
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -875,17 +875,17 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
@@ -905,7 +905,7 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -920,17 +920,17 @@
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104">
@@ -940,7 +940,7 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -960,12 +960,12 @@
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -995,7 +995,7 @@
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
@@ -1010,17 +1010,17 @@
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122">
@@ -1050,7 +1050,7 @@
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="128">
@@ -1065,7 +1065,7 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131">
@@ -1080,7 +1080,7 @@
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134">
@@ -1105,7 +1105,7 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -1115,22 +1115,22 @@
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="144">
@@ -1145,12 +1145,12 @@
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -1160,17 +1160,17 @@
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152">
@@ -1185,7 +1185,7 @@
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="155">

</xml_diff>